<commit_message>
Initial commit - force replace with local state
</commit_message>
<xml_diff>
--- a/CuttingParameterVerifier/wwwroot/samples/sample.xlsx
+++ b/CuttingParameterVerifier/wwwroot/samples/sample.xlsx
@@ -40,6 +40,9 @@
     <x:t>Tool Type (Carbide/HSS/PCD)</x:t>
   </x:si>
   <x:si>
+    <x:t>Machining Type (Conventional/HSM)</x:t>
+  </x:si>
+  <x:si>
     <x:t>Finish Type (Finish / Controlled Roughing / Free Roughing)</x:t>
   </x:si>
   <x:si>
@@ -76,49 +79,46 @@
     <x:t>Approach / Plunge Feed (mm/min)</x:t>
   </x:si>
   <x:si>
-    <x:t>Strategy Type</x:t>
-  </x:si>
-  <x:si>
     <x:t>Operation Name</x:t>
   </x:si>
   <x:si>
     <x:t/>
   </x:si>
   <x:si>
-    <x:t>Aluminum</x:t>
+    <x:t>Aluminium</x:t>
   </x:si>
   <x:si>
     <x:t>EM10</x:t>
   </x:si>
   <x:si>
-    <x:t>End milling</x:t>
+    <x:t>End Milling</x:t>
   </x:si>
   <x:si>
     <x:t>Carbide</x:t>
   </x:si>
   <x:si>
-    <x:t>Finishing</x:t>
-  </x:si>
-  <x:si>
     <x:t>Conventional</x:t>
   </x:si>
   <x:si>
+    <x:t>Finish</x:t>
+  </x:si>
+  <x:si>
     <x:t>Finish floor</x:t>
   </x:si>
   <x:si>
     <x:t>Finish wall</x:t>
   </x:si>
   <x:si>
-    <x:t>Steel</x:t>
-  </x:si>
-  <x:si>
     <x:t>EM12</x:t>
   </x:si>
   <x:si>
-    <x:t>Roughing</x:t>
+    <x:t>Controlled Roughing</x:t>
   </x:si>
   <x:si>
     <x:t>Rough pocket</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Free Roughing</x:t>
   </x:si>
   <x:si>
     <x:t>Invalid row demo</x:t>
@@ -483,19 +483,19 @@
     <x:col min="6" max="6" width="17.424911" style="0" customWidth="1"/>
     <x:col min="7" max="7" width="11.282054" style="0" customWidth="1"/>
     <x:col min="8" max="8" width="27.139196" style="0" customWidth="1"/>
-    <x:col min="9" max="9" width="53.282054" style="0" customWidth="1"/>
-    <x:col min="10" max="10" width="18.853482" style="0" customWidth="1"/>
-    <x:col min="11" max="11" width="22.996339" style="0" customWidth="1"/>
-    <x:col min="12" max="12" width="24.567768" style="0" customWidth="1"/>
-    <x:col min="13" max="13" width="21.424911" style="0" customWidth="1"/>
-    <x:col min="14" max="14" width="19.853482" style="0" customWidth="1"/>
-    <x:col min="15" max="15" width="20.996339" style="0" customWidth="1"/>
-    <x:col min="16" max="16" width="29.567768" style="0" customWidth="1"/>
-    <x:col min="17" max="17" width="16.710625" style="0" customWidth="1"/>
-    <x:col min="18" max="18" width="11.424911" style="0" customWidth="1"/>
-    <x:col min="19" max="19" width="16.567768" style="0" customWidth="1"/>
-    <x:col min="20" max="20" width="31.996339" style="0" customWidth="1"/>
-    <x:col min="21" max="21" width="13.282054" style="0" customWidth="1"/>
+    <x:col min="9" max="9" width="34.282054" style="0" customWidth="1"/>
+    <x:col min="10" max="10" width="53.282054" style="0" customWidth="1"/>
+    <x:col min="11" max="11" width="18.853482" style="0" customWidth="1"/>
+    <x:col min="12" max="12" width="22.996339" style="0" customWidth="1"/>
+    <x:col min="13" max="13" width="24.567768" style="0" customWidth="1"/>
+    <x:col min="14" max="14" width="21.424911" style="0" customWidth="1"/>
+    <x:col min="15" max="15" width="19.853482" style="0" customWidth="1"/>
+    <x:col min="16" max="16" width="20.996339" style="0" customWidth="1"/>
+    <x:col min="17" max="17" width="29.567768" style="0" customWidth="1"/>
+    <x:col min="18" max="18" width="16.710625" style="0" customWidth="1"/>
+    <x:col min="19" max="19" width="11.424911" style="0" customWidth="1"/>
+    <x:col min="20" max="20" width="16.567768" style="0" customWidth="1"/>
+    <x:col min="21" max="21" width="31.996339" style="0" customWidth="1"/>
     <x:col min="22" max="22" width="16.424911" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -595,33 +595,33 @@
       <x:c r="I2" s="0" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="J2" s="0">
+      <x:c r="J2" s="0" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="K2" s="0">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="K2" s="0">
+      <x:c r="L2" s="0">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="L2" s="0">
+      <x:c r="M2" s="0">
         <x:v>2400</x:v>
       </x:c>
-      <x:c r="M2" s="0">
+      <x:c r="N2" s="0">
         <x:v>12000</x:v>
       </x:c>
-      <x:c r="N2" s="0">
+      <x:c r="O2" s="0">
         <x:v>1.5</x:v>
       </x:c>
-      <x:c r="O2" s="0">
+      <x:c r="P2" s="0">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="P2" s="0">
+      <x:c r="Q2" s="0">
         <x:v>0.12</x:v>
       </x:c>
-      <x:c r="Q2" s="0">
+      <x:c r="R2" s="0">
         <x:v>600</x:v>
       </x:c>
-      <x:c r="R2" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="S2" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
@@ -629,7 +629,7 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="U2" s="0" t="s">
-        <x:v>28</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="V2" s="0" t="s">
         <x:v>29</x:v>
@@ -663,33 +663,33 @@
       <x:c r="I3" s="0" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="J3" s="0">
+      <x:c r="J3" s="0" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="K3" s="0">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="K3" s="0">
+      <x:c r="L3" s="0">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="L3" s="0">
+      <x:c r="M3" s="0">
         <x:v>2400</x:v>
       </x:c>
-      <x:c r="M3" s="0">
+      <x:c r="N3" s="0">
         <x:v>12000</x:v>
       </x:c>
-      <x:c r="N3" s="0">
+      <x:c r="O3" s="0">
         <x:v>1.5</x:v>
       </x:c>
-      <x:c r="O3" s="0">
+      <x:c r="P3" s="0">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="P3" s="0">
+      <x:c r="Q3" s="0">
         <x:v>0.35</x:v>
       </x:c>
-      <x:c r="Q3" s="0">
+      <x:c r="R3" s="0">
         <x:v>600</x:v>
       </x:c>
-      <x:c r="R3" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="S3" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
@@ -697,7 +697,7 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="U3" s="0" t="s">
-        <x:v>28</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="V3" s="0" t="s">
         <x:v>30</x:v>
@@ -714,13 +714,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="E4" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="F4" s="0" t="s">
         <x:v>31</x:v>
-      </x:c>
-      <x:c r="E4" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="F4" s="0" t="s">
-        <x:v>32</x:v>
       </x:c>
       <x:c r="G4" s="0" t="s">
         <x:v>25</x:v>
@@ -729,46 +729,46 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="I4" s="0" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="J4" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="K4" s="0">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="L4" s="0">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="M4" s="0">
+        <x:v>3600</x:v>
+      </x:c>
+      <x:c r="N4" s="0">
+        <x:v>9000</x:v>
+      </x:c>
+      <x:c r="O4" s="0">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="P4" s="0">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="Q4" s="0">
+        <x:v>0.08</x:v>
+      </x:c>
+      <x:c r="R4" s="0">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="S4" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="T4" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="U4" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="V4" s="0" t="s">
         <x:v>33</x:v>
-      </x:c>
-      <x:c r="J4" s="0">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="K4" s="0">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="L4" s="0">
-        <x:v>3600</x:v>
-      </x:c>
-      <x:c r="M4" s="0">
-        <x:v>9000</x:v>
-      </x:c>
-      <x:c r="N4" s="0">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="O4" s="0">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="P4" s="0">
-        <x:v>0.08</x:v>
-      </x:c>
-      <x:c r="Q4" s="0">
-        <x:v>400</x:v>
-      </x:c>
-      <x:c r="R4" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="S4" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="T4" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="U4" s="0" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="V4" s="0" t="s">
-        <x:v>34</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:22">
@@ -782,7 +782,7 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="E5" s="0" t="s">
         <x:v>22</x:v>
@@ -799,27 +799,27 @@
       <x:c r="I5" s="0" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="J5" s="0">
+      <x:c r="J5" s="0" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="K5" s="0">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="K5" s="0">
+      <x:c r="L5" s="0">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="L5" s="0">
+      <x:c r="M5" s="0">
         <x:v>2400</x:v>
       </x:c>
-      <x:c r="M5" s="0">
+      <x:c r="N5" s="0">
         <x:v>12000</x:v>
       </x:c>
-      <x:c r="N5" s="0">
+      <x:c r="O5" s="0">
         <x:v>1.5</x:v>
       </x:c>
-      <x:c r="O5" s="0">
+      <x:c r="P5" s="0">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="P5" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="Q5" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
@@ -833,7 +833,7 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="U5" s="0" t="s">
-        <x:v>28</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="V5" s="0" t="s">
         <x:v>35</x:v>

</xml_diff>